<commit_message>
Agregando permisos en esapño
</commit_message>
<xml_diff>
--- a/storage/app/utils/Permissions.xlsx
+++ b/storage/app/utils/Permissions.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\crm.atalaya\storage\app\utils\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97CFB5DB-C4BF-4FCD-950D-22286B126754}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C66A2C24-7026-48FB-AFD1-48044999FDCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="171">
   <si>
     <t>name</t>
   </si>
@@ -372,9 +372,6 @@
     <t>id</t>
   </si>
   <si>
-    <t>dashboard.list</t>
-  </si>
-  <si>
     <t>Permite visualizar la pantalla de dashboard</t>
   </si>
   <si>
@@ -430,6 +427,117 @@
   </si>
   <si>
     <t>El usuario podrá listar todos los proyectos. Si esta desactivado, solo puede ver sus asignados.</t>
+  </si>
+  <si>
+    <t>beauty</t>
+  </si>
+  <si>
+    <t>Todos</t>
+  </si>
+  <si>
+    <t>Ver</t>
+  </si>
+  <si>
+    <t>Agregar</t>
+  </si>
+  <si>
+    <t>Actualizar</t>
+  </si>
+  <si>
+    <t>Eliminar</t>
+  </si>
+  <si>
+    <t>Convertir en cliente</t>
+  </si>
+  <si>
+    <t>Cambiar estado</t>
+  </si>
+  <si>
+    <t>Actualizar contraseña</t>
+  </si>
+  <si>
+    <t>Estados</t>
+  </si>
+  <si>
+    <t>Agregar pagos</t>
+  </si>
+  <si>
+    <t>Actualizar pagos</t>
+  </si>
+  <si>
+    <t>Eliminar pagos</t>
+  </si>
+  <si>
+    <t>Agregar notas</t>
+  </si>
+  <si>
+    <t>Eliminar notas</t>
+  </si>
+  <si>
+    <t>Actualizar notas</t>
+  </si>
+  <si>
+    <t>Ver todos</t>
+  </si>
+  <si>
+    <t>model_name</t>
+  </si>
+  <si>
+    <t>Usuarios</t>
+  </si>
+  <si>
+    <t>Lead</t>
+  </si>
+  <si>
+    <t>Tablas</t>
+  </si>
+  <si>
+    <t>Permisos</t>
+  </si>
+  <si>
+    <t>Roles</t>
+  </si>
+  <si>
+    <t>Clientes</t>
+  </si>
+  <si>
+    <t>Leads</t>
+  </si>
+  <si>
+    <t>Cliente</t>
+  </si>
+  <si>
+    <t>Proyectos</t>
+  </si>
+  <si>
+    <t>Tipos</t>
+  </si>
+  <si>
+    <t>Proyecto</t>
+  </si>
+  <si>
+    <t>Pagos</t>
+  </si>
+  <si>
+    <t>Whatsapp</t>
+  </si>
+  <si>
+    <t>Configuraciones</t>
+  </si>
+  <si>
+    <t>Dashboard</t>
+  </si>
+  <si>
+    <t>Procesos</t>
+  </si>
+  <si>
+    <t>Poryectos</t>
+  </si>
+  <si>
+    <t>dashboard.projects</t>
+  </si>
+  <si>
+    <t>dashboard.leads</t>
   </si>
 </sst>
 </file>
@@ -753,15 +861,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1313F201-150F-4349-81B7-2BFCC09F2BD3}">
-  <dimension ref="A1:C68"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="84.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="22.7109375" customWidth="1"/>
+    <col min="5" max="5" width="84.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>114</v>
       </c>
@@ -769,737 +878,1153 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
+        <v>151</v>
+      </c>
+      <c r="D1" t="s">
+        <v>134</v>
+      </c>
+      <c r="E1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="E2" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="E3" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="E4" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="E5" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="E6" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="E7" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="E8" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="E9" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="E10" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="E11" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="E12" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="E13" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="E14" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="E15" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="E16" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="E17" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="E18" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="E19" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="E20" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="E21" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="E22" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="E23" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="E24" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="E25" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="E26" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C27" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="E27" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C28" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="E28" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="E29" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C30" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="E30" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="E31" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="E32" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C33" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="E33" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C34" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="E34" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C35" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="E35" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C36" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="E36" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C37" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="E37" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C38" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="E38" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C39" t="s">
+      <c r="C39" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="E39" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C40" t="s">
+      <c r="C40" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="E40" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C41" t="s">
+      <c r="C41" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="E41" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C42" t="s">
+      <c r="C42" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="E42" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C43" t="s">
+      <c r="C43" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="E43" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C44" t="s">
+      <c r="C44" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="E44" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C45" t="s">
+      <c r="C45" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="E45" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C46" t="s">
+      <c r="C46" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="E46" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C47" t="s">
+      <c r="C47" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="E47" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C48" t="s">
+      <c r="C48" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E48" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C49" t="s">
+      <c r="C49" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="E49" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C50" t="s">
+      <c r="C50" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="E50" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C51" t="s">
+      <c r="C51" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="E51" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>51</v>
       </c>
       <c r="B52" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C52" t="s">
+      <c r="C52" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="E52" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>52</v>
       </c>
       <c r="B53" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C53" t="s">
+      <c r="C53" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="E53" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>53</v>
       </c>
       <c r="B54" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C54" t="s">
+      <c r="C54" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="E54" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>54</v>
       </c>
       <c r="B55" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C55" t="s">
+      <c r="C55" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="E55" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>55</v>
       </c>
       <c r="B56" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C56" t="s">
+      <c r="C56" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="E56" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>56</v>
       </c>
       <c r="B57" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C57" t="s">
+      <c r="C57" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="E57" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>57</v>
       </c>
       <c r="B58" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="E58" t="s">
         <v>115</v>
       </c>
-      <c r="C58" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>58</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="C59" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+        <v>116</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="E59" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>59</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="C60" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="E60" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>60</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="C61" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="E61" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>61</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="C62" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+        <v>119</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="E62" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>62</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="C63" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+        <v>124</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="E63" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>63</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="C64" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C64" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="D64" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="E64" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>64</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="C65" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+        <v>127</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="D65" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="E65" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>65</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="C66" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+        <v>128</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="E66" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>66</v>
       </c>
       <c r="B67" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="D67" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="E67" t="s">
         <v>133</v>
       </c>
-      <c r="C67" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B68" s="1"/>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>57</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="D68" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="E68" t="s">
+        <v>115</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>